<commit_message>
adding plots, making as well fluorine comparison, as well if targeting could be rematched, answer nope cant be
</commit_message>
<xml_diff>
--- a/data/Chemical_table.xlsx
+++ b/data/Chemical_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inl-my.sharepoint.com/personal/meggie_krymowski_inl_gov/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meggie/Documents/MoltenSaltPropnet/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="116" documentId="8_{096C9E9E-33D3-B140-A6A9-BCBF2ACFD81B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7CF8164-F0E2-4A4E-8DC5-6D3717D03772}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C25AEC7-7E44-6D4B-8EB2-5CB22AD8416B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2480" yWindow="2120" windowWidth="20660" windowHeight="16960" xr2:uid="{6B23358E-95BA-7240-92EA-D47DA79C2B10}"/>
+    <workbookView xWindow="1360" yWindow="500" windowWidth="17580" windowHeight="15800" xr2:uid="{6B23358E-95BA-7240-92EA-D47DA79C2B10}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3105,7 +3105,7 @@
       <c r="S58" s="5"/>
       <c r="T58" s="5"/>
     </row>
-    <row r="59" spans="1:20" ht="18" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
@@ -3129,7 +3129,9 @@
       <c r="I59" s="2">
         <v>1.85</v>
       </c>
-      <c r="J59" s="2"/>
+      <c r="J59" s="2">
+        <v>1.96</v>
+      </c>
       <c r="K59" s="2">
         <v>534.4</v>
       </c>
@@ -3167,7 +3169,9 @@
       <c r="I60" s="2">
         <v>1.85</v>
       </c>
-      <c r="J60" s="2"/>
+      <c r="J60" s="2">
+        <v>1.95</v>
+      </c>
       <c r="K60" s="2">
         <v>527</v>
       </c>
@@ -3205,7 +3209,9 @@
       <c r="I61" s="2">
         <v>1.85</v>
       </c>
-      <c r="J61" s="2"/>
+      <c r="J61" s="2">
+        <v>1.94</v>
+      </c>
       <c r="K61" s="2">
         <v>533.1</v>
       </c>
@@ -3243,7 +3249,9 @@
       <c r="I62" s="2">
         <v>1.85</v>
       </c>
-      <c r="J62" s="2"/>
+      <c r="J62" s="2">
+        <v>1.93</v>
+      </c>
       <c r="K62" s="2">
         <v>540</v>
       </c>
@@ -3281,7 +3289,9 @@
       <c r="I63" s="2">
         <v>1.85</v>
       </c>
-      <c r="J63" s="2"/>
+      <c r="J63" s="2">
+        <v>1.92</v>
+      </c>
       <c r="K63" s="2">
         <v>544.5</v>
       </c>
@@ -3319,7 +3329,9 @@
       <c r="I64" s="2">
         <v>1.85</v>
       </c>
-      <c r="J64" s="2"/>
+      <c r="J64" s="2">
+        <v>1.92</v>
+      </c>
       <c r="K64" s="2">
         <v>547.1</v>
       </c>
@@ -3357,7 +3369,9 @@
       <c r="I65" s="2">
         <v>1.8</v>
       </c>
-      <c r="J65" s="2"/>
+      <c r="J65" s="2">
+        <v>1.91</v>
+      </c>
       <c r="K65" s="2">
         <v>593.4</v>
       </c>
@@ -3395,7 +3409,9 @@
       <c r="I66" s="2">
         <v>1.75</v>
       </c>
-      <c r="J66" s="2"/>
+      <c r="J66" s="2">
+        <v>1.9</v>
+      </c>
       <c r="K66" s="2">
         <v>565.79999999999995</v>
       </c>
@@ -3433,7 +3449,9 @@
       <c r="I67" s="2">
         <v>1.75</v>
       </c>
-      <c r="J67" s="2"/>
+      <c r="J67" s="2">
+        <v>1.89</v>
+      </c>
       <c r="K67" s="2">
         <v>573</v>
       </c>
@@ -3471,7 +3489,9 @@
       <c r="I68" s="2">
         <v>1.75</v>
       </c>
-      <c r="J68" s="2"/>
+      <c r="J68" s="2">
+        <v>1.88</v>
+      </c>
       <c r="K68" s="2">
         <v>581</v>
       </c>
@@ -3509,7 +3529,9 @@
       <c r="I69" s="2">
         <v>1.75</v>
       </c>
-      <c r="J69" s="2"/>
+      <c r="J69" s="2">
+        <v>1.88</v>
+      </c>
       <c r="K69" s="2">
         <v>589.29999999999995</v>
       </c>
@@ -3547,7 +3569,9 @@
       <c r="I70" s="2">
         <v>1.75</v>
       </c>
-      <c r="J70" s="2"/>
+      <c r="J70" s="2">
+        <v>1.87</v>
+      </c>
       <c r="K70" s="2">
         <v>596.70000000000005</v>
       </c>
@@ -3585,7 +3609,9 @@
       <c r="I71" s="2">
         <v>1.75</v>
       </c>
-      <c r="J71" s="2"/>
+      <c r="J71" s="2">
+        <v>1.87</v>
+      </c>
       <c r="K71" s="2">
         <v>603.4</v>
       </c>
@@ -4143,7 +4169,9 @@
       <c r="I85" s="2">
         <v>1.9</v>
       </c>
-      <c r="J85" s="2"/>
+      <c r="J85" s="2">
+        <v>1.98</v>
+      </c>
       <c r="K85" s="2">
         <v>812.1</v>
       </c>
@@ -4181,7 +4209,9 @@
       <c r="I86" s="2">
         <v>1.27</v>
       </c>
-      <c r="J86" s="2"/>
+      <c r="J86" s="2">
+        <v>2.02</v>
+      </c>
       <c r="K86" s="2">
         <v>899.00300000000004</v>
       </c>
@@ -4253,7 +4283,9 @@
       <c r="G88" s="4"/>
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
-      <c r="J88" s="2"/>
+      <c r="J88" s="2">
+        <v>2.23</v>
+      </c>
       <c r="K88" s="2">
         <v>393</v>
       </c>
@@ -4289,7 +4321,9 @@
       <c r="I89" s="2">
         <v>2.15</v>
       </c>
-      <c r="J89" s="2"/>
+      <c r="J89" s="2">
+        <v>2.0099999999999998</v>
+      </c>
       <c r="K89" s="2">
         <v>509.3</v>
       </c>
@@ -4327,7 +4361,9 @@
       <c r="I90" s="2">
         <v>1.95</v>
       </c>
-      <c r="J90" s="2"/>
+      <c r="J90" s="2">
+        <v>2.15</v>
+      </c>
       <c r="K90" s="2">
         <v>499</v>
       </c>
@@ -4365,7 +4401,9 @@
       <c r="I91" s="2">
         <v>1.8</v>
       </c>
-      <c r="J91" s="2"/>
+      <c r="J91" s="2">
+        <v>2.06</v>
+      </c>
       <c r="K91" s="2">
         <v>587</v>
       </c>
@@ -4403,7 +4441,9 @@
       <c r="I92" s="2">
         <v>1.8</v>
       </c>
-      <c r="J92" s="2"/>
+      <c r="J92" s="2">
+        <v>2</v>
+      </c>
       <c r="K92" s="2">
         <v>568</v>
       </c>
@@ -4441,7 +4481,9 @@
       <c r="I93" s="2">
         <v>1.75</v>
       </c>
-      <c r="J93" s="2"/>
+      <c r="J93" s="2">
+        <v>1.96</v>
+      </c>
       <c r="K93" s="2">
         <v>597.6</v>
       </c>
@@ -4477,7 +4519,9 @@
       <c r="I94" s="2">
         <v>1.75</v>
       </c>
-      <c r="J94" s="2"/>
+      <c r="J94" s="2">
+        <v>1.9</v>
+      </c>
       <c r="K94" s="2">
         <v>604.5</v>
       </c>
@@ -4513,7 +4557,9 @@
       <c r="I95" s="2">
         <v>1.75</v>
       </c>
-      <c r="J95" s="2"/>
+      <c r="J95" s="2">
+        <v>1.87</v>
+      </c>
       <c r="K95" s="2">
         <v>584.70000000000005</v>
       </c>
@@ -4549,7 +4595,9 @@
       <c r="I96" s="2">
         <v>1.75</v>
       </c>
-      <c r="J96" s="2"/>
+      <c r="J96" s="2">
+        <v>1.8</v>
+      </c>
       <c r="K96" s="2">
         <v>578</v>
       </c>
@@ -4575,7 +4623,9 @@
       </c>
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
-      <c r="J97" s="2"/>
+      <c r="J97" s="2">
+        <v>1.69</v>
+      </c>
       <c r="K97" s="2">
         <v>581</v>
       </c>

</xml_diff>